<commit_message>
Great Run: 22 nouvelles cellules finishers (2016-2025)
Source: raceresults.greatrun.org (Playwright batch scraper)
Events: Great North/South/Manchester/Birmingham/Bristol/Scottish Run

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
+++ b/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
@@ -8965,6 +8965,18 @@
           <t>x</t>
         </is>
       </c>
+      <c r="U62" t="n">
+        <v>26057</v>
+      </c>
+      <c r="V62" t="n">
+        <v>17172</v>
+      </c>
+      <c r="W62" t="n">
+        <v>18700</v>
+      </c>
+      <c r="X62" t="n">
+        <v>18258</v>
+      </c>
       <c r="Y62" t="inlineStr">
         <is>
           <t>-</t>
@@ -9094,6 +9106,15 @@
           <t>x</t>
         </is>
       </c>
+      <c r="V63" t="n">
+        <v>5787</v>
+      </c>
+      <c r="W63" t="n">
+        <v>4811</v>
+      </c>
+      <c r="X63" t="n">
+        <v>4521</v>
+      </c>
       <c r="Y63" t="inlineStr">
         <is>
           <t>-</t>
@@ -9141,6 +9162,18 @@
           <t>x</t>
         </is>
       </c>
+      <c r="U64" t="n">
+        <v>7088</v>
+      </c>
+      <c r="V64" t="n">
+        <v>7476</v>
+      </c>
+      <c r="W64" t="n">
+        <v>7030</v>
+      </c>
+      <c r="X64" t="n">
+        <v>6828</v>
+      </c>
       <c r="Y64" t="inlineStr">
         <is>
           <t>-</t>
@@ -10376,6 +10409,9 @@
       <c r="S77" t="n">
         <v>41615</v>
       </c>
+      <c r="T77" t="n">
+        <v>40906</v>
+      </c>
       <c r="U77" t="n">
         <v>41615</v>
       </c>
@@ -18480,6 +18516,15 @@
           <t>x</t>
         </is>
       </c>
+      <c r="T169" t="n">
+        <v>2719</v>
+      </c>
+      <c r="U169" t="n">
+        <v>3282</v>
+      </c>
+      <c r="V169" t="n">
+        <v>2968</v>
+      </c>
       <c r="Y169" t="inlineStr">
         <is>
           <t>-</t>
@@ -18724,6 +18769,18 @@
           <t>x</t>
         </is>
       </c>
+      <c r="U172" t="n">
+        <v>13079</v>
+      </c>
+      <c r="V172" t="n">
+        <v>8885</v>
+      </c>
+      <c r="W172" t="n">
+        <v>7898</v>
+      </c>
+      <c r="X172" t="n">
+        <v>7867</v>
+      </c>
       <c r="Y172" t="inlineStr">
         <is>
           <t>-</t>
@@ -18927,6 +18984,18 @@
           <t>x</t>
         </is>
       </c>
+      <c r="U174" t="n">
+        <v>9681</v>
+      </c>
+      <c r="V174" t="n">
+        <v>11189</v>
+      </c>
+      <c r="W174" t="n">
+        <v>10644</v>
+      </c>
+      <c r="X174" t="n">
+        <v>10170</v>
+      </c>
       <c r="Y174" t="inlineStr">
         <is>
           <t>-</t>
@@ -19014,6 +19083,18 @@
         <is>
           <t>AJ Bell Great South Run</t>
         </is>
+      </c>
+      <c r="U176" t="n">
+        <v>15642</v>
+      </c>
+      <c r="V176" t="n">
+        <v>16305</v>
+      </c>
+      <c r="W176" t="n">
+        <v>15840</v>
+      </c>
+      <c r="X176" t="n">
+        <v>15979</v>
       </c>
       <c r="Y176" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Great Run: injection finale — 49 cellules finishers (scrape complet)
Source: raceresults.greatrun.org (Playwright, 293 events scrapes)
Couverture: Great North/South/Manchester/Birmingham/Bristol/Scottish Run
Annees: 2007-2025 selon les events

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
+++ b/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
@@ -8965,6 +8965,24 @@
           <t>x</t>
         </is>
       </c>
+      <c r="N62" t="n">
+        <v>26938</v>
+      </c>
+      <c r="O62" t="n">
+        <v>27009</v>
+      </c>
+      <c r="P62" t="n">
+        <v>27796</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>29295</v>
+      </c>
+      <c r="R62" t="n">
+        <v>27803</v>
+      </c>
+      <c r="S62" t="n">
+        <v>27715</v>
+      </c>
       <c r="U62" t="n">
         <v>26057</v>
       </c>
@@ -10403,9 +10421,24 @@
       <c r="L77" t="n">
         <v>35777</v>
       </c>
+      <c r="M77" t="n">
+        <v>37127</v>
+      </c>
+      <c r="N77" t="n">
+        <v>37602</v>
+      </c>
       <c r="O77" t="n">
         <v>39459</v>
       </c>
+      <c r="P77" t="n">
+        <v>37526</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>40068</v>
+      </c>
+      <c r="R77" t="n">
+        <v>40737</v>
+      </c>
       <c r="S77" t="n">
         <v>41615</v>
       </c>
@@ -18516,6 +18549,21 @@
           <t>x</t>
         </is>
       </c>
+      <c r="N169" t="n">
+        <v>7856</v>
+      </c>
+      <c r="O169" t="n">
+        <v>6846</v>
+      </c>
+      <c r="Q169" t="n">
+        <v>4713</v>
+      </c>
+      <c r="R169" t="n">
+        <v>2340</v>
+      </c>
+      <c r="S169" t="n">
+        <v>2981</v>
+      </c>
       <c r="T169" t="n">
         <v>2719</v>
       </c>
@@ -18769,6 +18817,18 @@
           <t>x</t>
         </is>
       </c>
+      <c r="P172" t="n">
+        <v>11449</v>
+      </c>
+      <c r="Q172" t="n">
+        <v>12862</v>
+      </c>
+      <c r="R172" t="n">
+        <v>14700</v>
+      </c>
+      <c r="S172" t="n">
+        <v>14614</v>
+      </c>
       <c r="U172" t="n">
         <v>13079</v>
       </c>
@@ -19083,6 +19143,27 @@
         <is>
           <t>AJ Bell Great South Run</t>
         </is>
+      </c>
+      <c r="M176" t="n">
+        <v>11681</v>
+      </c>
+      <c r="N176" t="n">
+        <v>13901</v>
+      </c>
+      <c r="O176" t="n">
+        <v>14919</v>
+      </c>
+      <c r="P176" t="n">
+        <v>16178</v>
+      </c>
+      <c r="Q176" t="n">
+        <v>17048</v>
+      </c>
+      <c r="R176" t="n">
+        <v>16483</v>
+      </c>
+      <c r="S176" t="n">
+        <v>16043</v>
       </c>
       <c r="U176" t="n">
         <v>15642</v>

</xml_diff>